<commit_message>
Ajuste na planilha + html base
</commit_message>
<xml_diff>
--- a/planilha_base.xlsx
+++ b/planilha_base.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d562c6c8c4e36d0e/Área de Trabalho/Programação/Projetos/supplier_automation/Versao_Antiga_Streamilt/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d562c6c8c4e36d0e/Área de Trabalho/Programação/Projetos/supplier_automation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="7" documentId="11_2B59D2BFD3D05612737B271159A688B4553DE260" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0104BF8E-ECF1-4C84-84A7-9E3CFDA9E01B}"/>
+  <xr:revisionPtr revIDLastSave="8" documentId="11_2B59D2BFD3D05612737B271159A688B4553DE260" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5C379EC7-BC1E-4BE3-AD34-CAA2A2096D80}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,9 +27,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="29">
   <si>
-    <t>Admin</t>
-  </si>
-  <si>
     <t>Colaborador</t>
   </si>
   <si>
@@ -112,6 +109,9 @@
   </si>
   <si>
     <t>Gabriel Alves</t>
+  </si>
+  <si>
+    <t>Solicitante</t>
   </si>
 </sst>
 </file>
@@ -119,7 +119,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="&quot;R$&quot;\ #,##0.00"/>
+    <numFmt numFmtId="164" formatCode="&quot;R$&quot;\ #,##0.00"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -175,7 +175,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -486,27 +486,27 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" t="s">
         <v>5</v>
-      </c>
-      <c r="B2" t="s">
-        <v>6</v>
       </c>
       <c r="C2">
         <v>1001</v>
@@ -515,15 +515,15 @@
         <v>1500</v>
       </c>
       <c r="E2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C3">
         <v>1002</v>
@@ -532,15 +532,15 @@
         <v>1800</v>
       </c>
       <c r="E3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B4" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C4">
         <v>1003</v>
@@ -549,15 +549,15 @@
         <v>2200</v>
       </c>
       <c r="E4" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C5">
         <v>1004</v>
@@ -566,15 +566,15 @@
         <v>1600</v>
       </c>
       <c r="E5" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C6">
         <v>1005</v>
@@ -583,15 +583,15 @@
         <v>1900</v>
       </c>
       <c r="E6" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B7" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C7">
         <v>1006</v>
@@ -600,15 +600,15 @@
         <v>2100</v>
       </c>
       <c r="E7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B8" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C8">
         <v>1007</v>
@@ -617,15 +617,15 @@
         <v>1750</v>
       </c>
       <c r="E8" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B9" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C9">
         <v>1008</v>
@@ -634,15 +634,15 @@
         <v>2300</v>
       </c>
       <c r="E9" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B10" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C10">
         <v>1009</v>
@@ -651,15 +651,15 @@
         <v>1650</v>
       </c>
       <c r="E10" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B11" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C11">
         <v>1010</v>
@@ -668,15 +668,15 @@
         <v>2000</v>
       </c>
       <c r="E11" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B12" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C12">
         <v>1011</v>
@@ -685,15 +685,15 @@
         <v>1850</v>
       </c>
       <c r="E12" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B13" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C13">
         <v>1012</v>
@@ -702,15 +702,15 @@
         <v>2400</v>
       </c>
       <c r="E13" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B14" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C14">
         <v>1013</v>
@@ -719,15 +719,15 @@
         <v>1700</v>
       </c>
       <c r="E14" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B15" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C15">
         <v>1014</v>
@@ -736,15 +736,15 @@
         <v>2250</v>
       </c>
       <c r="E15" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B16" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C16">
         <v>1015</v>
@@ -753,15 +753,15 @@
         <v>1950</v>
       </c>
       <c r="E16" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B17" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C17">
         <v>1016</v>
@@ -770,15 +770,15 @@
         <v>2100</v>
       </c>
       <c r="E17" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B18" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C18">
         <v>1017</v>
@@ -787,15 +787,15 @@
         <v>1800</v>
       </c>
       <c r="E18" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B19" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C19">
         <v>1018</v>
@@ -804,15 +804,15 @@
         <v>2350</v>
       </c>
       <c r="E19" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B20" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C20">
         <v>1019</v>
@@ -821,15 +821,15 @@
         <v>1550</v>
       </c>
       <c r="E20" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B21" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C21">
         <v>1020</v>
@@ -838,7 +838,7 @@
         <v>2200</v>
       </c>
       <c r="E21" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>